<commit_message>
doc(plannification) : revoir et changer certaines durées conformément à la discussion avec le prof
[10][Done]
</commit_message>
<xml_diff>
--- a/doc/T294-planif-NeoJonathan.xlsx
+++ b/doc/T294-planif-NeoJonathan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pe40boh\Documents\Github\P_Web_294-Passion_lecture-Vue.js\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB065F11-1B26-4A7D-92E0-9DEDF951711A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86250B43-977D-4520-9C91-2B4281E64DBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -893,16 +893,16 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>25</c:v>
+                  <c:v>40</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>8</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>10</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>8</c:v>
@@ -2009,11 +2009,11 @@
         <v>15</v>
       </c>
       <c r="B17" s="26">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C17" s="20" t="str">
         <f t="shared" si="0"/>
-        <v>7.94%</v>
+        <v>3.17%</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="21" x14ac:dyDescent="0.35">
@@ -2021,11 +2021,11 @@
         <v>17</v>
       </c>
       <c r="B18" s="26">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="C18" s="18" t="str">
         <f t="shared" si="0"/>
-        <v>39.68%</v>
+        <v>63.49%</v>
       </c>
       <c r="D18" s="24"/>
     </row>
@@ -2034,11 +2034,11 @@
         <v>18</v>
       </c>
       <c r="B19" s="25">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C19" s="18" t="str">
         <f t="shared" si="0"/>
-        <v>12.7%</v>
+        <v>3.17%</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="21" x14ac:dyDescent="0.35">
@@ -2046,11 +2046,11 @@
         <v>19</v>
       </c>
       <c r="B20" s="26">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C20" s="20" t="str">
         <f t="shared" si="0"/>
-        <v>15.87%</v>
+        <v>6.35%</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="21" x14ac:dyDescent="0.35">

</xml_diff>